<commit_message>
manually excluded high freq C_xi_M picks, reran all with 100db filt
</commit_message>
<xml_diff>
--- a/results/soae_T_xi [int 100ms, bw=10p max, kaiser, df=50hz, rip=50db, crop=200hz, tau=500ms, hop_psd=250ms, nfft=None, win=hann].xlsx
+++ b/results/soae_T_xi [int 100ms, bw=10p max, kaiser, df=50hz, rip=50db, crop=200hz, tau=500ms, hop_psd=250ms, nfft=None, win=hann].xlsx
@@ -495,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>2658.705600883819</v>
+        <v>2658.705600880234</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -503,13 +503,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.01338849374789224</v>
+        <v>0.01619283719572547</v>
       </c>
       <c r="F2" t="n">
-        <v>10.09595357963647</v>
+        <v>10.09595355218707</v>
       </c>
       <c r="G2" t="n">
-        <v>4.317159094940021e-11</v>
+        <v>4.317159098743067e-11</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -538,7 +538,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>2658.705600883819</v>
+        <v>2658.705600880234</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -546,13 +546,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.01195116321449315</v>
+        <v>0.01446773296688147</v>
       </c>
       <c r="F3" t="n">
-        <v>10.09595357963647</v>
+        <v>10.09595355218707</v>
       </c>
       <c r="G3" t="n">
-        <v>4.317159094940021e-11</v>
+        <v>4.317159098743067e-11</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -581,7 +581,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>2804.068192067681</v>
+        <v>2804.06819206768</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -589,13 +589,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.02214317339481274</v>
+        <v>0.04993469816766517</v>
       </c>
       <c r="F4" t="n">
-        <v>3.099453846677615</v>
+        <v>3.09945385050024</v>
       </c>
       <c r="G4" t="n">
-        <v>2.801276045222655e-10</v>
+        <v>2.80127604286006e-10</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>2804.068192067681</v>
+        <v>2804.06819206768</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -632,13 +632,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.02039588339399511</v>
+        <v>0.04316684485268042</v>
       </c>
       <c r="F5" t="n">
-        <v>3.099453846677615</v>
+        <v>3.09945385050024</v>
       </c>
       <c r="G5" t="n">
-        <v>2.801276045222655e-10</v>
+        <v>2.80127604286006e-10</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>3220.800685291518</v>
+        <v>3220.800685291393</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.02474343572062819</v>
+        <v>0.09214802723446526</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8253318416870419</v>
+        <v>0.8253318426568844</v>
       </c>
       <c r="G6" t="n">
-        <v>1.897717189203859e-08</v>
+        <v>1.897717186856505e-08</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>3220.800685291518</v>
+        <v>3220.800685291393</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.02479214358139931</v>
+        <v>0.09280728164220288</v>
       </c>
       <c r="F7" t="n">
-        <v>0.8253318416870419</v>
+        <v>0.8253318426568844</v>
       </c>
       <c r="G7" t="n">
-        <v>1.897717189203859e-08</v>
+        <v>1.897717186856505e-08</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>3862.816359448726</v>
+        <v>3862.81635944896</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.0233570188302103</v>
+        <v>0.06480081213377525</v>
       </c>
       <c r="F8" t="n">
-        <v>2.212581609714611</v>
+        <v>2.212581609474567</v>
       </c>
       <c r="G8" t="n">
-        <v>1.143648050607118e-09</v>
+        <v>1.143648050677205e-09</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>3862.816359448726</v>
+        <v>3862.81635944896</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -804,13 +804,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.02250134938673089</v>
+        <v>0.06151187352007523</v>
       </c>
       <c r="F9" t="n">
-        <v>2.212581609714611</v>
+        <v>2.212581609474567</v>
       </c>
       <c r="G9" t="n">
-        <v>1.143648050607118e-09</v>
+        <v>1.143648050677205e-09</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>1297.253631950494</v>
+        <v>1297.253631949539</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -847,13 +847,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.02102405163160167</v>
+        <v>0.04589945799093244</v>
       </c>
       <c r="F10" t="n">
-        <v>1.30683405833951</v>
+        <v>1.306834054289299</v>
       </c>
       <c r="G10" t="n">
-        <v>3.769498660414696e-10</v>
+        <v>3.769498669948313e-10</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>1297.253631950494</v>
+        <v>1297.253631949539</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -890,13 +890,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.0204856764975675</v>
+        <v>0.05077690059357349</v>
       </c>
       <c r="F11" t="n">
-        <v>1.30683405833951</v>
+        <v>1.306834054289299</v>
       </c>
       <c r="G11" t="n">
-        <v>3.769498660414696e-10</v>
+        <v>3.769498669948313e-10</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>2340.356482943926</v>
+        <v>2340.356482942609</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -933,13 +933,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.02470281360534473</v>
+        <v>0.09241433289912161</v>
       </c>
       <c r="F12" t="n">
-        <v>1.226981091050554</v>
+        <v>1.226981092761272</v>
       </c>
       <c r="G12" t="n">
-        <v>5.938820762633677e-09</v>
+        <v>5.938820756495993e-09</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>2340.356482943926</v>
+        <v>2340.356482942609</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -976,13 +976,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.0247906823492055</v>
+        <v>0.09353214688264222</v>
       </c>
       <c r="F13" t="n">
-        <v>1.226981091050554</v>
+        <v>1.226981092761272</v>
       </c>
       <c r="G13" t="n">
-        <v>5.938820762633677e-09</v>
+        <v>5.938820756495993e-09</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>3400.668518752738</v>
+        <v>3400.668518752385</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1019,13 +1019,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.02107665578697443</v>
+        <v>0.04322100602032249</v>
       </c>
       <c r="F14" t="n">
-        <v>2.396894498172528</v>
+        <v>2.396894500224019</v>
       </c>
       <c r="G14" t="n">
-        <v>4.965598255067872e-11</v>
+        <v>4.965598254691534e-11</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>3400.668518752738</v>
+        <v>3400.668518752385</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1062,13 +1062,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.01955678060268487</v>
+        <v>0.03957684908204129</v>
       </c>
       <c r="F15" t="n">
-        <v>2.396894498172528</v>
+        <v>2.396894500224019</v>
       </c>
       <c r="G15" t="n">
-        <v>4.965598255067872e-11</v>
+        <v>4.965598254691534e-11</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>8309.972638555715</v>
+        <v>8309.972638555882</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1105,13 +1105,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.02463904621551546</v>
+        <v>0.08753068768056256</v>
       </c>
       <c r="F16" t="n">
-        <v>1.618801452987563</v>
+        <v>1.618801456042487</v>
       </c>
       <c r="G16" t="n">
-        <v>2.563162317917372e-08</v>
+        <v>2.563162315852645e-08</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>8309.972638555715</v>
+        <v>8309.972638555882</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1148,13 +1148,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.0237855480349503</v>
+        <v>0.07912607409348177</v>
       </c>
       <c r="F17" t="n">
-        <v>1.618801452987563</v>
+        <v>1.618801456042487</v>
       </c>
       <c r="G17" t="n">
-        <v>2.563162317917372e-08</v>
+        <v>2.563162315852645e-08</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
         <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>732.9916816689899</v>
+        <v>732.9916816689882</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1191,13 +1191,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.02293958452000703</v>
+        <v>0.07178557274843962</v>
       </c>
       <c r="F18" t="n">
-        <v>0.8820415848355398</v>
+        <v>0.8820415846920716</v>
       </c>
       <c r="G18" t="n">
-        <v>5.146264616172274e-09</v>
+        <v>5.146264616172276e-09</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1226,7 +1226,7 @@
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>732.9916816689899</v>
+        <v>732.9916816689882</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1234,13 +1234,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.02268328707217256</v>
+        <v>0.07474810791990068</v>
       </c>
       <c r="F19" t="n">
-        <v>0.8820415848355398</v>
+        <v>0.8820415846920716</v>
       </c>
       <c r="G19" t="n">
-        <v>5.146264616172274e-09</v>
+        <v>5.146264616172276e-09</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1269,7 +1269,7 @@
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>1634.57201879146</v>
+        <v>1634.572018791545</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.02162577202752154</v>
+        <v>0.04755422180411721</v>
       </c>
       <c r="F20" t="n">
-        <v>2.415225068045846</v>
+        <v>2.415225068705968</v>
       </c>
       <c r="G20" t="n">
-        <v>3.347713808061568e-10</v>
+        <v>3.347713806806397e-10</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>1634.57201879146</v>
+        <v>1634.572018791545</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1320,13 +1320,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.02054047099535065</v>
+        <v>0.04602282029369008</v>
       </c>
       <c r="F21" t="n">
-        <v>2.415225068045846</v>
+        <v>2.415225068705968</v>
       </c>
       <c r="G21" t="n">
-        <v>3.347713808061568e-10</v>
+        <v>3.347713806806397e-10</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1355,7 +1355,7 @@
         <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>2226.383938132359</v>
+        <v>2226.383938131224</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1363,13 +1363,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.02373211684563313</v>
+        <v>0.08028021677124433</v>
       </c>
       <c r="F22" t="n">
-        <v>1.28136768473695</v>
+        <v>1.281367686769816</v>
       </c>
       <c r="G22" t="n">
-        <v>1.331698353456759e-09</v>
+        <v>1.33169835208791e-09</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
         <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>2226.383938132359</v>
+        <v>2226.383938131224</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1406,13 +1406,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.02392682472802266</v>
+        <v>0.08394367912296258</v>
       </c>
       <c r="F23" t="n">
-        <v>1.28136768473695</v>
+        <v>1.281367686769816</v>
       </c>
       <c r="G23" t="n">
-        <v>1.331698353456759e-09</v>
+        <v>1.33169835208791e-09</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
         <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>3120.340914912985</v>
+        <v>3120.340914913273</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1449,13 +1449,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.01329364269285412</v>
+        <v>0.01531130739877217</v>
       </c>
       <c r="F24" t="n">
-        <v>10.05992015692969</v>
+        <v>10.05992016213009</v>
       </c>
       <c r="G24" t="n">
-        <v>3.327547521360905e-11</v>
+        <v>3.327547518404527e-11</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1484,7 +1484,7 @@
         <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>3120.340914912985</v>
+        <v>3120.340914913273</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1492,13 +1492,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.01153232667724684</v>
+        <v>0.01331343473168582</v>
       </c>
       <c r="F25" t="n">
-        <v>10.05992015692969</v>
+        <v>10.05992016213009</v>
       </c>
       <c r="G25" t="n">
-        <v>3.327547521360905e-11</v>
+        <v>3.327547518404527e-11</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1527,7 +1527,7 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>904.9407547044033</v>
+        <v>904.9407547043927</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1535,10 +1535,10 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.02277555132777851</v>
+        <v>0.06721317561278579</v>
       </c>
       <c r="F26" t="n">
-        <v>0.8440441283854054</v>
+        <v>0.8440441282866774</v>
       </c>
       <c r="G26" t="n">
         <v>5.520043013082024e-07</v>
@@ -1570,7 +1570,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>904.9407547044033</v>
+        <v>904.9407547043927</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1578,10 +1578,10 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.02255915134628286</v>
+        <v>0.07131676825730426</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8440441283854054</v>
+        <v>0.8440441282866774</v>
       </c>
       <c r="G27" t="n">
         <v>5.520043013082024e-07</v>
@@ -1613,7 +1613,7 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>1520.28126739245</v>
+        <v>1520.281267393959</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1621,13 +1621,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.02390369133254361</v>
+        <v>0.08156254170436035</v>
       </c>
       <c r="F28" t="n">
-        <v>1.25461465454959</v>
+        <v>1.254614652958397</v>
       </c>
       <c r="G28" t="n">
-        <v>3.486811568038311e-07</v>
+        <v>3.486811571447247e-07</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
         <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>1520.28126739245</v>
+        <v>1520.281267393959</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1664,13 +1664,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.0240436400339157</v>
+        <v>0.08521127830210458</v>
       </c>
       <c r="F29" t="n">
-        <v>1.25461465454959</v>
+        <v>1.254614652958397</v>
       </c>
       <c r="G29" t="n">
-        <v>3.486811568038311e-07</v>
+        <v>3.486811571447247e-07</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>2282.24851917037</v>
+        <v>2282.248519170488</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1707,13 +1707,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.02126931247804847</v>
+        <v>0.04017648026524131</v>
       </c>
       <c r="F30" t="n">
-        <v>4.481984427283572</v>
+        <v>4.481984426888731</v>
       </c>
       <c r="G30" t="n">
-        <v>2.437506213742745e-08</v>
+        <v>2.437506213825452e-08</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1742,7 +1742,7 @@
         <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>2282.24851917037</v>
+        <v>2282.248519170488</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1750,13 +1750,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.01967296457538953</v>
+        <v>0.03584219671184762</v>
       </c>
       <c r="F31" t="n">
-        <v>4.481984427283572</v>
+        <v>4.481984426888731</v>
       </c>
       <c r="G31" t="n">
-        <v>2.437506213742745e-08</v>
+        <v>2.437506213825452e-08</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1785,7 +1785,7 @@
         <v>3</v>
       </c>
       <c r="C32" t="n">
-        <v>6044.943088003415</v>
+        <v>6044.943088003487</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1793,13 +1793,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.02073766660490962</v>
+        <v>0.04158558444205579</v>
       </c>
       <c r="F32" t="n">
-        <v>1.621707514225389</v>
+        <v>1.621707514273231</v>
       </c>
       <c r="G32" t="n">
-        <v>2.512844909272361e-08</v>
+        <v>2.512844909276033e-08</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -1828,7 +1828,7 @@
         <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>6044.943088003415</v>
+        <v>6044.943088003487</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1836,13 +1836,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.01910616422779206</v>
+        <v>0.03761328834344413</v>
       </c>
       <c r="F33" t="n">
-        <v>1.621707514225389</v>
+        <v>1.621707514273231</v>
       </c>
       <c r="G33" t="n">
-        <v>2.512844909272361e-08</v>
+        <v>2.512844909276033e-08</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>1233.124123086937</v>
+        <v>1233.124123086702</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1879,13 +1879,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.01517263497583422</v>
+        <v>0.01795570188025535</v>
       </c>
       <c r="F34" t="n">
-        <v>11.88039216112336</v>
+        <v>11.8803921636882</v>
       </c>
       <c r="G34" t="n">
-        <v>9.671861630740103e-10</v>
+        <v>9.671861629676735e-10</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1914,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>1233.124123086937</v>
+        <v>1233.124123086702</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1922,13 +1922,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.01476618215578882</v>
+        <v>0.01763430339672063</v>
       </c>
       <c r="F35" t="n">
-        <v>11.88039216112336</v>
+        <v>11.8803921636882</v>
       </c>
       <c r="G35" t="n">
-        <v>9.671861630740103e-10</v>
+        <v>9.671861629676735e-10</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1957,7 +1957,7 @@
         <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>3111.790660208523</v>
+        <v>3111.790660196808</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1965,13 +1965,13 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.00373994024234344</v>
+        <v>0.004345318120719598</v>
       </c>
       <c r="F36" t="n">
-        <v>40.81661001733268</v>
+        <v>40.81661019133534</v>
       </c>
       <c r="G36" t="n">
-        <v>3.507570265881665e-10</v>
+        <v>3.507570270931431e-10</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2000,7 +2000,7 @@
         <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>3111.790660208523</v>
+        <v>3111.790660196808</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2008,13 +2008,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.003372543386907341</v>
+        <v>0.003838433455166207</v>
       </c>
       <c r="F37" t="n">
-        <v>40.81661001733268</v>
+        <v>40.81661019133534</v>
       </c>
       <c r="G37" t="n">
-        <v>3.507570265881665e-10</v>
+        <v>3.507570270931431e-10</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>3704.49737123546</v>
+        <v>3704.497371235483</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2051,13 +2051,13 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.01026138418936711</v>
+        <v>0.01144058070100376</v>
       </c>
       <c r="F38" t="n">
-        <v>19.05817478880967</v>
+        <v>19.05817478384657</v>
       </c>
       <c r="G38" t="n">
-        <v>4.267083315417213e-09</v>
+        <v>4.267083315442432e-09</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
         <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>3704.49737123546</v>
+        <v>3704.497371235483</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2094,13 +2094,13 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.01010186351521546</v>
+        <v>0.0112841362154434</v>
       </c>
       <c r="F39" t="n">
-        <v>19.05817478880967</v>
+        <v>19.05817478384657</v>
       </c>
       <c r="G39" t="n">
-        <v>4.267083315417213e-09</v>
+        <v>4.267083315442432e-09</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2129,7 +2129,7 @@
         <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>4500.984900280526</v>
+        <v>4500.984900283443</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2137,13 +2137,13 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.00491228866412795</v>
+        <v>0.005831056967114798</v>
       </c>
       <c r="F40" t="n">
-        <v>33.25889727068895</v>
+        <v>33.25889734469793</v>
       </c>
       <c r="G40" t="n">
-        <v>1.853307281611389e-10</v>
+        <v>1.853307282346105e-10</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2172,7 +2172,7 @@
         <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>4500.984900280526</v>
+        <v>4500.984900283443</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2180,13 +2180,13 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.004742749991719378</v>
+        <v>0.005560237765161611</v>
       </c>
       <c r="F41" t="n">
-        <v>33.25889727068895</v>
+        <v>33.25889734469793</v>
       </c>
       <c r="G41" t="n">
-        <v>1.853307281611389e-10</v>
+        <v>1.853307282346105e-10</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2215,7 +2215,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>966.296209019041</v>
+        <v>966.2962090192465</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2223,13 +2223,13 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.009867491005898007</v>
+        <v>0.01101229643282171</v>
       </c>
       <c r="F42" t="n">
-        <v>16.38970636450469</v>
+        <v>16.38970637248534</v>
       </c>
       <c r="G42" t="n">
-        <v>6.199727859154702e-10</v>
+        <v>6.199727859341858e-10</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2258,7 +2258,7 @@
         <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>966.296209019041</v>
+        <v>966.2962090192465</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2266,13 +2266,13 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.009485482172376212</v>
+        <v>0.01061481699804798</v>
       </c>
       <c r="F43" t="n">
-        <v>16.38970636450469</v>
+        <v>16.38970637248534</v>
       </c>
       <c r="G43" t="n">
-        <v>6.199727859154702e-10</v>
+        <v>6.199727859341858e-10</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>2268.980486823418</v>
+        <v>2268.980486795794</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2309,13 +2309,13 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.004701449017125424</v>
+        <v>0.005365915472914974</v>
       </c>
       <c r="F44" t="n">
-        <v>30.52335914219278</v>
+        <v>30.52335899097242</v>
       </c>
       <c r="G44" t="n">
-        <v>2.21881720560141e-10</v>
+        <v>2.218817204193758e-10</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2344,7 +2344,7 @@
         <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>2268.980486823418</v>
+        <v>2268.980486795794</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2352,13 +2352,13 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.004222341715638375</v>
+        <v>0.004903504274438586</v>
       </c>
       <c r="F45" t="n">
-        <v>30.52335914219278</v>
+        <v>30.52335899097242</v>
       </c>
       <c r="G45" t="n">
-        <v>2.21881720560141e-10</v>
+        <v>2.218817204193758e-10</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>3152.979193945399</v>
+        <v>3152.979193945613</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2395,13 +2395,13 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.00797883573499507</v>
+        <v>0.008776512963732067</v>
       </c>
       <c r="F46" t="n">
-        <v>24.19350635585815</v>
+        <v>24.19350636189434</v>
       </c>
       <c r="G46" t="n">
-        <v>5.273689268421645e-09</v>
+        <v>5.273689267512965e-09</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2430,7 +2430,7 @@
         <v>1</v>
       </c>
       <c r="C47" t="n">
-        <v>3152.979193945399</v>
+        <v>3152.979193945613</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2438,13 +2438,13 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.007878088854375617</v>
+        <v>0.008566030336961114</v>
       </c>
       <c r="F47" t="n">
-        <v>24.19350635585815</v>
+        <v>24.19350636189434</v>
       </c>
       <c r="G47" t="n">
-        <v>5.273689268421645e-09</v>
+        <v>5.273689267512965e-09</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
         <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>3942.312467070839</v>
+        <v>3942.312467066556</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2481,13 +2481,13 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.00435583699939475</v>
+        <v>0.005125583134892512</v>
       </c>
       <c r="F48" t="n">
-        <v>42.70877088698131</v>
+        <v>42.70877068563502</v>
       </c>
       <c r="G48" t="n">
-        <v>1.492955403893206e-09</v>
+        <v>1.492955402385597e-09</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -2516,7 +2516,7 @@
         <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>3942.312467070839</v>
+        <v>3942.312467066556</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2524,13 +2524,13 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.00431673040823008</v>
+        <v>0.005035543468726513</v>
       </c>
       <c r="F49" t="n">
-        <v>42.70877088698131</v>
+        <v>42.70877068563502</v>
       </c>
       <c r="G49" t="n">
-        <v>1.492955403893206e-09</v>
+        <v>1.492955402385597e-09</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         <v>2</v>
       </c>
       <c r="C50" t="n">
-        <v>1725.77246271569</v>
+        <v>1725.772462710338</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2567,13 +2567,13 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.006221654036319391</v>
+        <v>0.007244950228959879</v>
       </c>
       <c r="F50" t="n">
-        <v>22.02734009913382</v>
+        <v>22.02734034403161</v>
       </c>
       <c r="G50" t="n">
-        <v>3.8334456361479e-10</v>
+        <v>3.833445630578505e-10</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
         <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>1725.77246271569</v>
+        <v>1725.772462710338</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2610,13 +2610,13 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.005689119327560682</v>
+        <v>0.006680025507169288</v>
       </c>
       <c r="F51" t="n">
-        <v>22.02734009913382</v>
+        <v>22.02734034403161</v>
       </c>
       <c r="G51" t="n">
-        <v>3.8334456361479e-10</v>
+        <v>3.833445630578505e-10</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>2</v>
       </c>
       <c r="C52" t="n">
-        <v>2175.217037016602</v>
+        <v>2175.217037016691</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2653,13 +2653,13 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.01320298115643232</v>
+        <v>0.01537020561047446</v>
       </c>
       <c r="F52" t="n">
-        <v>14.68264699292376</v>
+        <v>14.68264699299626</v>
       </c>
       <c r="G52" t="n">
-        <v>3.372737978265115e-09</v>
+        <v>3.372737978453659e-09</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2688,7 +2688,7 @@
         <v>2</v>
       </c>
       <c r="C53" t="n">
-        <v>2175.217037016602</v>
+        <v>2175.217037016691</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2696,13 +2696,13 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.01306503381126856</v>
+        <v>0.0150719801513951</v>
       </c>
       <c r="F53" t="n">
-        <v>14.68264699292376</v>
+        <v>14.68264699299626</v>
       </c>
       <c r="G53" t="n">
-        <v>3.372737978265115e-09</v>
+        <v>3.372737978453659e-09</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
         <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>3112.955084064267</v>
+        <v>3112.955084064253</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2739,13 +2739,13 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.007492255416200839</v>
+        <v>0.008085157476641378</v>
       </c>
       <c r="F54" t="n">
-        <v>26.12811731054386</v>
+        <v>26.1281172770193</v>
       </c>
       <c r="G54" t="n">
-        <v>2.373397884964904e-09</v>
+        <v>2.373397884407087e-09</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2774,7 +2774,7 @@
         <v>2</v>
       </c>
       <c r="C55" t="n">
-        <v>3112.955084064267</v>
+        <v>3112.955084064253</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2782,13 +2782,13 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.007448373140906589</v>
+        <v>0.008037017294446013</v>
       </c>
       <c r="F55" t="n">
-        <v>26.12811731054386</v>
+        <v>26.1281172770193</v>
       </c>
       <c r="G55" t="n">
-        <v>2.373397884964904e-09</v>
+        <v>2.373397884407087e-09</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v>2</v>
       </c>
       <c r="C56" t="n">
-        <v>3478.093550335875</v>
+        <v>3478.093550335324</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.007625343380389936</v>
+        <v>0.00839168791114219</v>
       </c>
       <c r="F56" t="n">
-        <v>24.43832251578529</v>
+        <v>24.43832250664904</v>
       </c>
       <c r="G56" t="n">
-        <v>1.666962751209387e-09</v>
+        <v>1.666962751163243e-09</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2860,7 +2860,7 @@
         <v>2</v>
       </c>
       <c r="C57" t="n">
-        <v>3478.093550335875</v>
+        <v>3478.093550335324</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2868,13 +2868,13 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.007425985702961762</v>
+        <v>0.008088190797932396</v>
       </c>
       <c r="F57" t="n">
-        <v>24.43832251578529</v>
+        <v>24.43832250664904</v>
       </c>
       <c r="G57" t="n">
-        <v>1.666962751209387e-09</v>
+        <v>1.666962751163243e-09</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -2903,7 +2903,7 @@
         <v>3</v>
       </c>
       <c r="C58" t="n">
-        <v>1792.591402055871</v>
+        <v>1792.591402057709</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2911,13 +2911,13 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.007895239723442067</v>
+        <v>0.009037738992722965</v>
       </c>
       <c r="F58" t="n">
-        <v>25.14257025556138</v>
+        <v>25.14257025564731</v>
       </c>
       <c r="G58" t="n">
-        <v>5.849111394182677e-10</v>
+        <v>5.849111392773192e-10</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
         <v>3</v>
       </c>
       <c r="C59" t="n">
-        <v>1792.591402055871</v>
+        <v>1792.591402057709</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2954,13 +2954,13 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.007391091340058374</v>
+        <v>0.008583097431505534</v>
       </c>
       <c r="F59" t="n">
-        <v>25.14257025556138</v>
+        <v>25.14257025564731</v>
       </c>
       <c r="G59" t="n">
-        <v>5.849111394182677e-10</v>
+        <v>5.849111392773192e-10</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
         <v>3</v>
       </c>
       <c r="C60" t="n">
-        <v>2141.987315973998</v>
+        <v>2141.987315972156</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2997,13 +2997,13 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.002887545295871246</v>
+        <v>0.003342262957582712</v>
       </c>
       <c r="F60" t="n">
-        <v>64.87424358314686</v>
+        <v>64.87424396895483</v>
       </c>
       <c r="G60" t="n">
-        <v>1.057816834562884e-10</v>
+        <v>1.05781683859114e-10</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -3032,7 +3032,7 @@
         <v>3</v>
       </c>
       <c r="C61" t="n">
-        <v>2141.987315973998</v>
+        <v>2141.987315972156</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3040,13 +3040,13 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.002594747748693942</v>
+        <v>0.003007403348800386</v>
       </c>
       <c r="F61" t="n">
-        <v>64.87424358314686</v>
+        <v>64.87424396895483</v>
       </c>
       <c r="G61" t="n">
-        <v>1.057816834562884e-10</v>
+        <v>1.05781683859114e-10</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         <v>3</v>
       </c>
       <c r="C62" t="n">
-        <v>2411.713690307367</v>
+        <v>2411.713690301313</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3083,13 +3083,13 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.00320094181218953</v>
+        <v>0.003841892013640759</v>
       </c>
       <c r="F62" t="n">
-        <v>48.24737097415694</v>
+        <v>48.24737092155696</v>
       </c>
       <c r="G62" t="n">
-        <v>6.382896709194328e-11</v>
+        <v>6.382896710760599e-11</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3118,7 +3118,7 @@
         <v>3</v>
       </c>
       <c r="C63" t="n">
-        <v>2411.713690307367</v>
+        <v>2411.713690301313</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3126,13 +3126,13 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.002861689124708259</v>
+        <v>0.003395288608305442</v>
       </c>
       <c r="F63" t="n">
-        <v>48.24737097415694</v>
+        <v>48.24737092155696</v>
       </c>
       <c r="G63" t="n">
-        <v>6.382896709194328e-11</v>
+        <v>6.382896710760599e-11</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
         <v>3</v>
       </c>
       <c r="C64" t="n">
-        <v>3047.241393740617</v>
+        <v>3047.241393754507</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3169,13 +3169,13 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.003528265687307975</v>
+        <v>0.003982502583665556</v>
       </c>
       <c r="F64" t="n">
-        <v>42.07107085886242</v>
+        <v>42.07107102770869</v>
       </c>
       <c r="G64" t="n">
-        <v>7.356289947329848e-11</v>
+        <v>7.356289959298675e-11</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
         <v>3</v>
       </c>
       <c r="C65" t="n">
-        <v>3047.241393740617</v>
+        <v>3047.241393754507</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3212,13 +3212,13 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.003103145812186566</v>
+        <v>0.003579927589809419</v>
       </c>
       <c r="F65" t="n">
-        <v>42.07107085886242</v>
+        <v>42.07107102770869</v>
       </c>
       <c r="G65" t="n">
-        <v>7.356289947329848e-11</v>
+        <v>7.356289959298675e-11</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>1346.541722579976</v>
+        <v>1346.541722553406</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.003726937272989729</v>
+        <v>0.004304911509268628</v>
       </c>
       <c r="F66" t="n">
-        <v>40.32418981350884</v>
+        <v>40.32418949488441</v>
       </c>
       <c r="G66" t="n">
-        <v>3.659803900682979e-11</v>
+        <v>3.659803894855202e-11</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
@@ -3290,7 +3290,7 @@
         <v>0</v>
       </c>
       <c r="C67" t="n">
-        <v>1346.541722579976</v>
+        <v>1346.541722553406</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3298,13 +3298,13 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.003371407653444637</v>
+        <v>0.003956226368134414</v>
       </c>
       <c r="F67" t="n">
-        <v>40.32418981350884</v>
+        <v>40.32418949488441</v>
       </c>
       <c r="G67" t="n">
-        <v>3.659803900682979e-11</v>
+        <v>3.659803894855202e-11</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
         <v>0</v>
       </c>
       <c r="C68" t="n">
-        <v>1782.753690589079</v>
+        <v>1782.753690595554</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3341,13 +3341,13 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.007253718598177967</v>
+        <v>0.008377438115076026</v>
       </c>
       <c r="F68" t="n">
-        <v>21.79457753296188</v>
+        <v>21.79457757467633</v>
       </c>
       <c r="G68" t="n">
-        <v>7.430242443755415e-11</v>
+        <v>7.430242442575194e-11</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -3376,7 +3376,7 @@
         <v>0</v>
       </c>
       <c r="C69" t="n">
-        <v>1782.753690589079</v>
+        <v>1782.753690595554</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3384,13 +3384,13 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>0.006732541622804819</v>
+        <v>0.007906181432659466</v>
       </c>
       <c r="F69" t="n">
-        <v>21.79457753296188</v>
+        <v>21.79457757467633</v>
       </c>
       <c r="G69" t="n">
-        <v>7.430242443755415e-11</v>
+        <v>7.430242442575194e-11</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -3419,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>3641.458414255485</v>
+        <v>3641.458414264404</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3427,13 +3427,13 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.004327707767644662</v>
+        <v>0.005139596617196733</v>
       </c>
       <c r="F70" t="n">
-        <v>35.27900030025856</v>
+        <v>35.27900051644691</v>
       </c>
       <c r="G70" t="n">
-        <v>2.276951422908099e-11</v>
+        <v>2.276951425078513e-11</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -3462,7 +3462,7 @@
         <v>0</v>
       </c>
       <c r="C71" t="n">
-        <v>3641.458414255485</v>
+        <v>3641.458414264404</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3470,13 +3470,13 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.00396632937270708</v>
+        <v>0.004632226374767556</v>
       </c>
       <c r="F71" t="n">
-        <v>35.27900030025856</v>
+        <v>35.27900051644691</v>
       </c>
       <c r="G71" t="n">
-        <v>2.276951422908099e-11</v>
+        <v>2.276951425078513e-11</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -3505,7 +3505,7 @@
         <v>0</v>
       </c>
       <c r="C72" t="n">
-        <v>4210.606778278299</v>
+        <v>4210.60677827836</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3513,13 +3513,13 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.01025461408632988</v>
+        <v>0.01205317017253553</v>
       </c>
       <c r="F72" t="n">
-        <v>15.48239600579577</v>
+        <v>15.48239598695274</v>
       </c>
       <c r="G72" t="n">
-        <v>3.761604213414296e-11</v>
+        <v>3.761604214434703e-11</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>4210.606778278299</v>
+        <v>4210.60677827836</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3556,13 +3556,13 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.009981751118988942</v>
+        <v>0.01203175499595989</v>
       </c>
       <c r="F73" t="n">
-        <v>15.48239600579577</v>
+        <v>15.48239598695274</v>
       </c>
       <c r="G73" t="n">
-        <v>3.761604213414296e-11</v>
+        <v>3.761604214434703e-11</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -3591,7 +3591,7 @@
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>1358.804474952999</v>
+        <v>1358.804474954195</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3599,10 +3599,10 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.005251492591661726</v>
+        <v>0.005887696057666738</v>
       </c>
       <c r="F74" t="n">
-        <v>26.01227643333035</v>
+        <v>26.01227642789845</v>
       </c>
       <c r="G74" t="n">
         <v>1.707056566304335e-11</v>
@@ -3634,7 +3634,7 @@
         <v>1</v>
       </c>
       <c r="C75" t="n">
-        <v>1358.804474952999</v>
+        <v>1358.804474954195</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3642,10 +3642,10 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.004601231394884948</v>
+        <v>0.005139333015065598</v>
       </c>
       <c r="F75" t="n">
-        <v>26.01227643333035</v>
+        <v>26.01227642789845</v>
       </c>
       <c r="G75" t="n">
         <v>1.707056566304335e-11</v>
@@ -3677,7 +3677,7 @@
         <v>1</v>
       </c>
       <c r="C76" t="n">
-        <v>1777.561135908246</v>
+        <v>1777.56113590488</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3685,13 +3685,13 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.00558011120332368</v>
+        <v>0.006156124842335765</v>
       </c>
       <c r="F76" t="n">
-        <v>24.55723343006592</v>
+        <v>24.55723338600139</v>
       </c>
       <c r="G76" t="n">
-        <v>2.28406500232103e-11</v>
+        <v>2.284065002447836e-11</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -3720,7 +3720,7 @@
         <v>1</v>
       </c>
       <c r="C77" t="n">
-        <v>1777.561135908246</v>
+        <v>1777.56113590488</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3728,13 +3728,13 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.004992944832327433</v>
+        <v>0.005509100717764075</v>
       </c>
       <c r="F77" t="n">
-        <v>24.55723343006592</v>
+        <v>24.55723338600139</v>
       </c>
       <c r="G77" t="n">
-        <v>2.28406500232103e-11</v>
+        <v>2.284065002447836e-11</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -3763,7 +3763,7 @@
         <v>1</v>
       </c>
       <c r="C78" t="n">
-        <v>3604.619040898234</v>
+        <v>3604.619040897909</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3771,13 +3771,13 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.007594383479081057</v>
+        <v>0.008372377315018281</v>
       </c>
       <c r="F78" t="n">
-        <v>23.55508939978257</v>
+        <v>23.555089386247</v>
       </c>
       <c r="G78" t="n">
-        <v>6.738722230488649e-11</v>
+        <v>6.738722231221811e-11</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -3806,7 +3806,7 @@
         <v>1</v>
       </c>
       <c r="C79" t="n">
-        <v>3604.619040898234</v>
+        <v>3604.619040897909</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3814,13 +3814,13 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.007114092375918404</v>
+        <v>0.007812964343873829</v>
       </c>
       <c r="F79" t="n">
-        <v>23.55508939978257</v>
+        <v>23.555089386247</v>
       </c>
       <c r="G79" t="n">
-        <v>6.738722230488649e-11</v>
+        <v>6.738722231221811e-11</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -3849,7 +3849,7 @@
         <v>1</v>
       </c>
       <c r="C80" t="n">
-        <v>4388.66998755417</v>
+        <v>4388.669987553901</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3857,13 +3857,13 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.004636944951928543</v>
+        <v>0.005503378682193936</v>
       </c>
       <c r="F80" t="n">
-        <v>30.94992804312051</v>
+        <v>30.94992821931555</v>
       </c>
       <c r="G80" t="n">
-        <v>1.198402805005504e-11</v>
+        <v>1.198402805938865e-11</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -3892,7 +3892,7 @@
         <v>1</v>
       </c>
       <c r="C81" t="n">
-        <v>4388.66998755417</v>
+        <v>4388.669987553901</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3900,13 +3900,13 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.004187323961586985</v>
+        <v>0.004895016679069444</v>
       </c>
       <c r="F81" t="n">
-        <v>30.94992804312051</v>
+        <v>30.94992821931555</v>
       </c>
       <c r="G81" t="n">
-        <v>1.198402805005504e-11</v>
+        <v>1.198402805938865e-11</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -3935,7 +3935,7 @@
         <v>2</v>
       </c>
       <c r="C82" t="n">
-        <v>1256.91613658691</v>
+        <v>1256.916136586966</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3943,13 +3943,13 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.009091230378911403</v>
+        <v>0.009945427089160736</v>
       </c>
       <c r="F82" t="n">
-        <v>17.11041971790514</v>
+        <v>17.11041974211544</v>
       </c>
       <c r="G82" t="n">
-        <v>4.581825436838118e-11</v>
+        <v>4.581825435534533e-11</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -3978,7 +3978,7 @@
         <v>2</v>
       </c>
       <c r="C83" t="n">
-        <v>1256.91613658691</v>
+        <v>1256.916136586966</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3986,13 +3986,13 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0.008267484268276891</v>
+        <v>0.009195537985459273</v>
       </c>
       <c r="F83" t="n">
-        <v>17.11041971790514</v>
+        <v>17.11041974211544</v>
       </c>
       <c r="G83" t="n">
-        <v>4.581825436838118e-11</v>
+        <v>4.581825435534533e-11</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -4021,7 +4021,7 @@
         <v>2</v>
       </c>
       <c r="C84" t="n">
-        <v>1689.76559169971</v>
+        <v>1689.765591700369</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -4029,10 +4029,10 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>0.005364159875899709</v>
+        <v>0.006172171532534934</v>
       </c>
       <c r="F84" t="n">
-        <v>25.09099687420753</v>
+        <v>25.09099671696914</v>
       </c>
       <c r="G84" t="n">
         <v>1.583280146603159e-11</v>
@@ -4064,7 +4064,7 @@
         <v>2</v>
       </c>
       <c r="C85" t="n">
-        <v>1689.76559169971</v>
+        <v>1689.765591700369</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -4072,10 +4072,10 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.004668509731518767</v>
+        <v>0.005554523714799353</v>
       </c>
       <c r="F85" t="n">
-        <v>25.09099687420753</v>
+        <v>25.09099671696914</v>
       </c>
       <c r="G85" t="n">
         <v>1.583280146603159e-11</v>
@@ -4107,7 +4107,7 @@
         <v>2</v>
       </c>
       <c r="C86" t="n">
-        <v>2565.453452588377</v>
+        <v>2565.453452577413</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -4115,13 +4115,13 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0.003063461175820288</v>
+        <v>0.003550695860228338</v>
       </c>
       <c r="F86" t="n">
-        <v>56.10647002579313</v>
+        <v>56.10647072185828</v>
       </c>
       <c r="G86" t="n">
-        <v>1.018124122957592e-11</v>
+        <v>1.018124129306755e-11</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -4150,7 +4150,7 @@
         <v>2</v>
       </c>
       <c r="C87" t="n">
-        <v>2565.453452588377</v>
+        <v>2565.453452577413</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -4158,13 +4158,13 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>0.002631364634691628</v>
+        <v>0.003065261752104785</v>
       </c>
       <c r="F87" t="n">
-        <v>56.10647002579313</v>
+        <v>56.10647072185828</v>
       </c>
       <c r="G87" t="n">
-        <v>1.018124122957592e-11</v>
+        <v>1.018124129306755e-11</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -4193,7 +4193,7 @@
         <v>2</v>
       </c>
       <c r="C88" t="n">
-        <v>3558.207975758685</v>
+        <v>3558.207975758281</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -4201,13 +4201,13 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.00646129301035952</v>
+        <v>0.007299373040289919</v>
       </c>
       <c r="F88" t="n">
-        <v>26.61131078072319</v>
+        <v>26.61131083407046</v>
       </c>
       <c r="G88" t="n">
-        <v>2.974314303249287e-11</v>
+        <v>2.974314302777163e-11</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -4236,7 +4236,7 @@
         <v>2</v>
       </c>
       <c r="C89" t="n">
-        <v>3558.207975758685</v>
+        <v>3558.207975758281</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>0.006074201518524538</v>
+        <v>0.006956472612081157</v>
       </c>
       <c r="F89" t="n">
-        <v>26.61131078072319</v>
+        <v>26.61131083407046</v>
       </c>
       <c r="G89" t="n">
-        <v>2.974314303249287e-11</v>
+        <v>2.974314302777163e-11</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -4279,7 +4279,7 @@
         <v>3</v>
       </c>
       <c r="C90" t="n">
-        <v>1251.380070750952</v>
+        <v>1251.380070751246</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4287,13 +4287,13 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>0.009446720234368589</v>
+        <v>0.0106850103491097</v>
       </c>
       <c r="F90" t="n">
-        <v>17.17910082708332</v>
+        <v>17.17910082644781</v>
       </c>
       <c r="G90" t="n">
-        <v>6.687451272124087e-11</v>
+        <v>6.687451272360359e-11</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -4322,7 +4322,7 @@
         <v>3</v>
       </c>
       <c r="C91" t="n">
-        <v>1251.380070750952</v>
+        <v>1251.380070751246</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4330,13 +4330,13 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.008745711907028641</v>
+        <v>0.009768250737280918</v>
       </c>
       <c r="F91" t="n">
-        <v>17.17910082708332</v>
+        <v>17.17910082644781</v>
       </c>
       <c r="G91" t="n">
-        <v>6.687451272124087e-11</v>
+        <v>6.687451272360359e-11</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -4365,7 +4365,7 @@
         <v>3</v>
       </c>
       <c r="C92" t="n">
-        <v>1485.47455592929</v>
+        <v>1485.474555923857</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4373,13 +4373,13 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.003602689498293962</v>
+        <v>0.004236428234354169</v>
       </c>
       <c r="F92" t="n">
-        <v>41.33077224631148</v>
+        <v>41.33077231855378</v>
       </c>
       <c r="G92" t="n">
-        <v>1.927134736616189e-11</v>
+        <v>1.927134739295641e-11</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
         <v>3</v>
       </c>
       <c r="C93" t="n">
-        <v>1485.47455592929</v>
+        <v>1485.474555923857</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4416,13 +4416,13 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.003149931714821035</v>
+        <v>0.003754138893107712</v>
       </c>
       <c r="F93" t="n">
-        <v>41.33077224631148</v>
+        <v>41.33077231855378</v>
       </c>
       <c r="G93" t="n">
-        <v>1.927134736616189e-11</v>
+        <v>1.927134739295641e-11</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -4451,7 +4451,7 @@
         <v>3</v>
       </c>
       <c r="C94" t="n">
-        <v>3221.719220257907</v>
+        <v>3221.719220271636</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4459,13 +4459,13 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.004490451738159812</v>
+        <v>0.005149149462053412</v>
       </c>
       <c r="F94" t="n">
-        <v>31.93359475693042</v>
+        <v>31.93359446629537</v>
       </c>
       <c r="G94" t="n">
-        <v>6.415294116942879e-12</v>
+        <v>6.415294109604703e-12</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -4494,7 +4494,7 @@
         <v>3</v>
       </c>
       <c r="C95" t="n">
-        <v>3221.719220257907</v>
+        <v>3221.719220271636</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4502,13 +4502,13 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>0.004021799389603826</v>
+        <v>0.004737902207628833</v>
       </c>
       <c r="F95" t="n">
-        <v>31.93359475693042</v>
+        <v>31.93359446629537</v>
       </c>
       <c r="G95" t="n">
-        <v>6.415294116942879e-12</v>
+        <v>6.415294109604703e-12</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -4537,7 +4537,7 @@
         <v>3</v>
       </c>
       <c r="C96" t="n">
-        <v>3584.49987011075</v>
+        <v>3584.499870105694</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4545,13 +4545,13 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>0.004846733626714205</v>
+        <v>0.005542884347363374</v>
       </c>
       <c r="F96" t="n">
-        <v>35.10352872377204</v>
+        <v>35.1035288170361</v>
       </c>
       <c r="G96" t="n">
-        <v>3.112263332790618e-11</v>
+        <v>3.112263333792322e-11</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -4580,7 +4580,7 @@
         <v>3</v>
       </c>
       <c r="C97" t="n">
-        <v>3584.49987011075</v>
+        <v>3584.499870105694</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4588,13 +4588,13 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>0.004383394792693165</v>
+        <v>0.004984991945041822</v>
       </c>
       <c r="F97" t="n">
-        <v>35.10352872377204</v>
+        <v>35.1035288170361</v>
       </c>
       <c r="G97" t="n">
-        <v>3.112263332790618e-11</v>
+        <v>3.112263333792322e-11</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
         <v>0</v>
       </c>
       <c r="C98" t="n">
-        <v>4343.968770688863</v>
+        <v>4343.968770693115</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4631,10 +4631,10 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0.002309045619922018</v>
+        <v>0.002742612235604423</v>
       </c>
       <c r="F98" t="n">
-        <v>70.42713647571071</v>
+        <v>70.42713629849885</v>
       </c>
       <c r="G98" t="n">
         <v>1.985614504899256e-13</v>
@@ -4666,7 +4666,7 @@
         <v>0</v>
       </c>
       <c r="C99" t="n">
-        <v>4343.968770688863</v>
+        <v>4343.968770693115</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4674,10 +4674,10 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>0.001991060102665277</v>
+        <v>0.002357756940811681</v>
       </c>
       <c r="F99" t="n">
-        <v>70.42713647571071</v>
+        <v>70.42713629849885</v>
       </c>
       <c r="G99" t="n">
         <v>1.985614504899256e-13</v>
@@ -4709,7 +4709,7 @@
         <v>0</v>
       </c>
       <c r="C100" t="n">
-        <v>5579.25028030521</v>
+        <v>5579.250280288047</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4717,13 +4717,13 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>0.003141669385428758</v>
+        <v>0.003721108502461276</v>
       </c>
       <c r="F100" t="n">
-        <v>48.09727917611898</v>
+        <v>48.09727907943265</v>
       </c>
       <c r="G100" t="n">
-        <v>3.754894706117401e-13</v>
+        <v>3.754894705158709e-13</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -4752,7 +4752,7 @@
         <v>0</v>
       </c>
       <c r="C101" t="n">
-        <v>5579.25028030521</v>
+        <v>5579.250280288047</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4760,13 +4760,13 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0.002726323787995442</v>
+        <v>0.003246781009563909</v>
       </c>
       <c r="F101" t="n">
-        <v>48.09727917611898</v>
+        <v>48.09727907943265</v>
       </c>
       <c r="G101" t="n">
-        <v>3.754894706117401e-13</v>
+        <v>3.754894705158709e-13</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -4795,7 +4795,7 @@
         <v>0</v>
       </c>
       <c r="C102" t="n">
-        <v>7456.556780554461</v>
+        <v>7456.556780530206</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4803,13 +4803,13 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>0.00325406484287731</v>
+        <v>0.003796977361887171</v>
       </c>
       <c r="F102" t="n">
-        <v>48.35560196622247</v>
+        <v>48.35560222806118</v>
       </c>
       <c r="G102" t="n">
-        <v>9.005871783377205e-13</v>
+        <v>9.005871802567054e-13</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -4838,7 +4838,7 @@
         <v>0</v>
       </c>
       <c r="C103" t="n">
-        <v>7456.556780554461</v>
+        <v>7456.556780530206</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4846,13 +4846,13 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>0.002871872175444953</v>
+        <v>0.003362907167913807</v>
       </c>
       <c r="F103" t="n">
-        <v>48.35560196622247</v>
+        <v>48.35560222806118</v>
       </c>
       <c r="G103" t="n">
-        <v>9.005871783377205e-13</v>
+        <v>9.005871802567054e-13</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -4881,7 +4881,7 @@
         <v>0</v>
       </c>
       <c r="C104" t="n">
-        <v>9030.433721340078</v>
+        <v>9030.433721344429</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4889,13 +4889,13 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>0.004335883556419119</v>
+        <v>0.004942050580719152</v>
       </c>
       <c r="F104" t="n">
-        <v>41.34715219631315</v>
+        <v>41.34715232351992</v>
       </c>
       <c r="G104" t="n">
-        <v>3.555680071586571e-12</v>
+        <v>3.55568007713164e-12</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -4924,7 +4924,7 @@
         <v>0</v>
       </c>
       <c r="C105" t="n">
-        <v>9030.433721340078</v>
+        <v>9030.433721344429</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4932,13 +4932,13 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>0.003843309740995608</v>
+        <v>0.004336315724308013</v>
       </c>
       <c r="F105" t="n">
-        <v>41.34715219631315</v>
+        <v>41.34715232351992</v>
       </c>
       <c r="G105" t="n">
-        <v>3.555680071586571e-12</v>
+        <v>3.55568007713164e-12</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -4967,7 +4967,7 @@
         <v>1</v>
       </c>
       <c r="C106" t="n">
-        <v>6840.972766591844</v>
+        <v>6840.972766602154</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4975,13 +4975,13 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>0.003144821569156814</v>
+        <v>0.003730418116833878</v>
       </c>
       <c r="F106" t="n">
-        <v>48.82276884010786</v>
+        <v>48.82276869525922</v>
       </c>
       <c r="G106" t="n">
-        <v>4.828196065042162e-13</v>
+        <v>4.828196055440911e-13</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -5010,7 +5010,7 @@
         <v>1</v>
       </c>
       <c r="C107" t="n">
-        <v>6840.972766591844</v>
+        <v>6840.972766602154</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -5018,13 +5018,13 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>0.002732493672434935</v>
+        <v>0.00324834567617055</v>
       </c>
       <c r="F107" t="n">
-        <v>48.82276884010786</v>
+        <v>48.82276869525922</v>
       </c>
       <c r="G107" t="n">
-        <v>4.828196065042162e-13</v>
+        <v>4.828196055440911e-13</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -5053,7 +5053,7 @@
         <v>1</v>
       </c>
       <c r="C108" t="n">
-        <v>7901.028542795753</v>
+        <v>7901.028542795319</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -5061,13 +5061,13 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>0.00469886952908061</v>
+        <v>0.00533067337344006</v>
       </c>
       <c r="F108" t="n">
-        <v>34.72295932312269</v>
+        <v>34.72295925128499</v>
       </c>
       <c r="G108" t="n">
-        <v>1.189062068220207e-12</v>
+        <v>1.189062068322416e-12</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v>1</v>
       </c>
       <c r="C109" t="n">
-        <v>7901.028542795753</v>
+        <v>7901.028542795319</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -5104,13 +5104,13 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>0.004118107577842785</v>
+        <v>0.004674528297641426</v>
       </c>
       <c r="F109" t="n">
-        <v>34.72295932312269</v>
+        <v>34.72295925128499</v>
       </c>
       <c r="G109" t="n">
-        <v>1.189062068220207e-12</v>
+        <v>1.189062068322416e-12</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -5139,7 +5139,7 @@
         <v>1</v>
       </c>
       <c r="C110" t="n">
-        <v>8846.195208391457</v>
+        <v>8846.19520838986</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -5147,13 +5147,13 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>0.004118270154199614</v>
+        <v>0.004785298419648373</v>
       </c>
       <c r="F110" t="n">
-        <v>43.26334015556915</v>
+        <v>43.26334017048392</v>
       </c>
       <c r="G110" t="n">
-        <v>2.335254089609143e-12</v>
+        <v>2.335254089590644e-12</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -5182,7 +5182,7 @@
         <v>1</v>
       </c>
       <c r="C111" t="n">
-        <v>8846.195208391457</v>
+        <v>8846.19520838986</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -5190,13 +5190,13 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>0.003602600868161113</v>
+        <v>0.00421648962688253</v>
       </c>
       <c r="F111" t="n">
-        <v>43.26334015556915</v>
+        <v>43.26334017048392</v>
       </c>
       <c r="G111" t="n">
-        <v>2.335254089609143e-12</v>
+        <v>2.335254089590644e-12</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -5225,7 +5225,7 @@
         <v>1</v>
       </c>
       <c r="C112" t="n">
-        <v>9783.556116822216</v>
+        <v>9783.556116786825</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -5233,13 +5233,13 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>0.001861531719711905</v>
+        <v>0.002241040299607083</v>
       </c>
       <c r="F112" t="n">
-        <v>91.0543750632585</v>
+        <v>91.05438059951148</v>
       </c>
       <c r="G112" t="n">
-        <v>1.085409814364765e-12</v>
+        <v>1.085409880004288e-12</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
@@ -5268,7 +5268,7 @@
         <v>1</v>
       </c>
       <c r="C113" t="n">
-        <v>9783.556116822216</v>
+        <v>9783.556116786825</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -5276,13 +5276,13 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>0.001617265929782431</v>
+        <v>0.001951957788754238</v>
       </c>
       <c r="F113" t="n">
-        <v>91.0543750632585</v>
+        <v>91.05438059951148</v>
       </c>
       <c r="G113" t="n">
-        <v>1.085409814364765e-12</v>
+        <v>1.085409880004288e-12</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
         <v>2</v>
       </c>
       <c r="C114" t="n">
-        <v>5622.683411663123</v>
+        <v>5622.683411661134</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -5319,13 +5319,13 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>0.005419958147782466</v>
+        <v>0.006149115379346184</v>
       </c>
       <c r="F114" t="n">
-        <v>29.1534451404782</v>
+        <v>29.15344518718943</v>
       </c>
       <c r="G114" t="n">
-        <v>1.307159835669512e-10</v>
+        <v>1.307159835869711e-10</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -5354,7 +5354,7 @@
         <v>2</v>
       </c>
       <c r="C115" t="n">
-        <v>5622.683411663123</v>
+        <v>5622.683411661134</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -5362,13 +5362,13 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>0.004731451375207111</v>
+        <v>0.005403416014047665</v>
       </c>
       <c r="F115" t="n">
-        <v>29.1534451404782</v>
+        <v>29.15344518718943</v>
       </c>
       <c r="G115" t="n">
-        <v>1.307159835669512e-10</v>
+        <v>1.307159835869711e-10</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
         <v>2</v>
       </c>
       <c r="C116" t="n">
-        <v>8098.504347864297</v>
+        <v>8098.50434786478</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -5405,13 +5405,13 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>0.003455577910051527</v>
+        <v>0.003998952423259975</v>
       </c>
       <c r="F116" t="n">
-        <v>49.72373807757332</v>
+        <v>49.72373786348046</v>
       </c>
       <c r="G116" t="n">
-        <v>2.153356701200664e-10</v>
+        <v>2.153356696819132e-10</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
@@ -5440,7 +5440,7 @@
         <v>2</v>
       </c>
       <c r="C117" t="n">
-        <v>8098.504347864297</v>
+        <v>8098.50434786478</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -5448,13 +5448,13 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>0.002993011482274934</v>
+        <v>0.003442731973587259</v>
       </c>
       <c r="F117" t="n">
-        <v>49.72373807757332</v>
+        <v>49.72373786348046</v>
       </c>
       <c r="G117" t="n">
-        <v>2.153356701200664e-10</v>
+        <v>2.153356696819132e-10</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -5483,7 +5483,7 @@
         <v>2</v>
       </c>
       <c r="C118" t="n">
-        <v>8486.629661786945</v>
+        <v>8486.629661785102</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -5491,13 +5491,13 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>0.009271376254818737</v>
+        <v>0.01075599354813443</v>
       </c>
       <c r="F118" t="n">
-        <v>19.85800756374371</v>
+        <v>19.85800760568668</v>
       </c>
       <c r="G118" t="n">
-        <v>7.360252862072354e-10</v>
+        <v>7.360252858797782e-10</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -5526,7 +5526,7 @@
         <v>2</v>
       </c>
       <c r="C119" t="n">
-        <v>8486.629661786945</v>
+        <v>8486.629661785102</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>0.008639559981426919</v>
+        <v>0.009982543076378643</v>
       </c>
       <c r="F119" t="n">
-        <v>19.85800756374371</v>
+        <v>19.85800760568668</v>
       </c>
       <c r="G119" t="n">
-        <v>7.360252862072354e-10</v>
+        <v>7.360252858797782e-10</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
@@ -5569,7 +5569,7 @@
         <v>2</v>
       </c>
       <c r="C120" t="n">
-        <v>9856.170123128086</v>
+        <v>9856.170123127897</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -5577,13 +5577,13 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>0.003537404137781667</v>
+        <v>0.004149742283513431</v>
       </c>
       <c r="F120" t="n">
-        <v>44.79676965174966</v>
+        <v>44.79676977747089</v>
       </c>
       <c r="G120" t="n">
-        <v>1.46067501429033e-10</v>
+        <v>1.460675015342739e-10</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
@@ -5612,7 +5612,7 @@
         <v>2</v>
       </c>
       <c r="C121" t="n">
-        <v>9856.170123128086</v>
+        <v>9856.170123127897</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -5620,13 +5620,13 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>0.003108772796239897</v>
+        <v>0.003711139080945708</v>
       </c>
       <c r="F121" t="n">
-        <v>44.79676965174966</v>
+        <v>44.79676977747089</v>
       </c>
       <c r="G121" t="n">
-        <v>1.46067501429033e-10</v>
+        <v>1.460675015342739e-10</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -5655,7 +5655,7 @@
         <v>3</v>
       </c>
       <c r="C122" t="n">
-        <v>5350.733987166818</v>
+        <v>5350.733987166514</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -5663,13 +5663,13 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>0.0019874017842229</v>
+        <v>0.00234290000527192</v>
       </c>
       <c r="F122" t="n">
-        <v>86.8513233141271</v>
+        <v>86.85132295553052</v>
       </c>
       <c r="G122" t="n">
-        <v>3.932146572144296e-11</v>
+        <v>3.932146572144297e-11</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
         <v>3</v>
       </c>
       <c r="C123" t="n">
-        <v>5350.733987166818</v>
+        <v>5350.733987166514</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5706,13 +5706,13 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>0.001689480608669042</v>
+        <v>0.001998175062770492</v>
       </c>
       <c r="F123" t="n">
-        <v>86.8513233141271</v>
+        <v>86.85132295553052</v>
       </c>
       <c r="G123" t="n">
-        <v>3.932146572144296e-11</v>
+        <v>3.932146572144297e-11</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
@@ -5741,7 +5741,7 @@
         <v>3</v>
       </c>
       <c r="C124" t="n">
-        <v>7182.136095056413</v>
+        <v>7182.136095056334</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5749,13 +5749,13 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>0.0221927133618091</v>
+        <v>0.04110683868157289</v>
       </c>
       <c r="F124" t="n">
-        <v>5.437958954940312</v>
+        <v>5.437958953595492</v>
       </c>
       <c r="G124" t="n">
-        <v>1.127045032891671e-08</v>
+        <v>1.127045032844483e-08</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
@@ -5784,7 +5784,7 @@
         <v>3</v>
       </c>
       <c r="C125" t="n">
-        <v>7182.136095056413</v>
+        <v>7182.136095056334</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5792,13 +5792,13 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>0.02134347610650427</v>
+        <v>0.03845907686688554</v>
       </c>
       <c r="F125" t="n">
-        <v>5.437958954940312</v>
+        <v>5.437958953595492</v>
       </c>
       <c r="G125" t="n">
-        <v>1.127045032891671e-08</v>
+        <v>1.127045032844483e-08</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
@@ -5827,7 +5827,7 @@
         <v>3</v>
       </c>
       <c r="C126" t="n">
-        <v>8447.007108264974</v>
+        <v>8447.007108267682</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5835,13 +5835,13 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>0.003309593673970049</v>
+        <v>0.003902242627650128</v>
       </c>
       <c r="F126" t="n">
-        <v>47.57406725471835</v>
+        <v>47.57406740201719</v>
       </c>
       <c r="G126" t="n">
-        <v>1.321469852555001e-10</v>
+        <v>1.321469853216139e-10</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -5870,7 +5870,7 @@
         <v>3</v>
       </c>
       <c r="C127" t="n">
-        <v>8447.007108264974</v>
+        <v>8447.007108267682</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -5878,13 +5878,13 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>0.002872841693285339</v>
+        <v>0.003331239802176662</v>
       </c>
       <c r="F127" t="n">
-        <v>47.57406725471835</v>
+        <v>47.57406740201719</v>
       </c>
       <c r="G127" t="n">
-        <v>1.321469852555001e-10</v>
+        <v>1.321469853216139e-10</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
@@ -5913,7 +5913,7 @@
         <v>3</v>
       </c>
       <c r="C128" t="n">
-        <v>9634.45516704175</v>
+        <v>9634.45516704174</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5921,13 +5921,13 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>0.01599681608458665</v>
+        <v>0.0193998623765043</v>
       </c>
       <c r="F128" t="n">
-        <v>11.3439055292692</v>
+        <v>11.3439055252793</v>
       </c>
       <c r="G128" t="n">
-        <v>3.808138262852559e-09</v>
+        <v>3.808138263015406e-09</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
@@ -5956,7 +5956,7 @@
         <v>3</v>
       </c>
       <c r="C129" t="n">
-        <v>9634.45516704175</v>
+        <v>9634.45516704174</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -5964,13 +5964,13 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>0.01504304570950625</v>
+        <v>0.01821758770856435</v>
       </c>
       <c r="F129" t="n">
-        <v>11.3439055292692</v>
+        <v>11.3439055252793</v>
       </c>
       <c r="G129" t="n">
-        <v>3.808138262852559e-09</v>
+        <v>3.808138263015406e-09</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>

</xml_diff>